<commit_message>
some more work on variables, descriptives, EFA and regressions
</commit_message>
<xml_diff>
--- a/data_frost.xlsx
+++ b/data_frost.xlsx
@@ -131,7 +131,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:FG100"/>
+  <dimension ref="A1:FG103"/>
   <cols>
     <col collapsed="false" hidden="false" max="1" min="1" style="0" customWidth="true" width="8"/>
     <col collapsed="false" hidden="false" max="2" min="2" style="0" customWidth="true" width="20"/>
@@ -2216,10 +2216,10 @@
         <v>39</v>
       </c>
       <c r="FF3" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="FG3" s="4" t="n">
-        <v>1.55</v>
+        <v>1.58</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="4">
@@ -2424,7 +2424,7 @@
         <v>100</v>
       </c>
       <c r="FG4" s="4" t="n">
-        <v>1.54</v>
+        <v>1.67</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="5">
@@ -2629,7 +2629,7 @@
         <v>100</v>
       </c>
       <c r="FG5" s="4" t="n">
-        <v>1.97</v>
+        <v>2.13</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="6">
@@ -2808,7 +2808,7 @@
       <c r="EU6" s="1"/>
       <c r="EV6" s="1"/>
       <c r="EW6" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="EX6" s="3"/>
       <c r="EY6" s="3" t="n">
@@ -3253,7 +3253,7 @@
         <v>4</v>
       </c>
       <c r="FG7" s="4" t="n">
-        <v>0.69</v>
+        <v>0.7</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="8">
@@ -3716,7 +3716,7 @@
         <v>2</v>
       </c>
       <c r="FG8" s="4" t="n">
-        <v>1.55</v>
+        <v>1.56</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="9">
@@ -4095,7 +4095,7 @@
         <v>4</v>
       </c>
       <c r="EW9" s="1" t="n">
-        <v>342</v>
+        <v>382</v>
       </c>
       <c r="EX9" s="3"/>
       <c r="EY9" s="3" t="n">
@@ -4125,7 +4125,7 @@
         <v>2</v>
       </c>
       <c r="FG9" s="4" t="n">
-        <v>1.29</v>
+        <v>1.3</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="10">
@@ -4592,7 +4592,7 @@
         <v>2</v>
       </c>
       <c r="FG10" s="4" t="n">
-        <v>0.93</v>
+        <v>0.94</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="11">
@@ -5027,7 +5027,7 @@
         <v>2</v>
       </c>
       <c r="FG11" s="4" t="n">
-        <v>1.2</v>
+        <v>1.21</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="12">
@@ -5446,7 +5446,7 @@
         <v>4</v>
       </c>
       <c r="FG12" s="4" t="n">
-        <v>1.45</v>
+        <v>1.46</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="13">
@@ -5853,7 +5853,7 @@
         <v>3</v>
       </c>
       <c r="FG13" s="4" t="n">
-        <v>1.23</v>
+        <v>1.24</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="14">
@@ -6521,7 +6521,7 @@
         <v>100</v>
       </c>
       <c r="FG15" s="4" t="n">
-        <v>1.09</v>
+        <v>1.21</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="16">
@@ -6700,7 +6700,7 @@
       <c r="EU16" s="1"/>
       <c r="EV16" s="1"/>
       <c r="EW16" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="EX16" s="3"/>
       <c r="EY16" s="3" t="n">
@@ -6726,7 +6726,7 @@
         <v>100</v>
       </c>
       <c r="FG16" s="4" t="n">
-        <v>0.32</v>
+        <v>0.34</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="17">
@@ -7596,7 +7596,7 @@
         <v>2</v>
       </c>
       <c r="FG18" s="4" t="n">
-        <v>1.52</v>
+        <v>1.53</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="19">
@@ -8055,7 +8055,7 @@
         <v>2</v>
       </c>
       <c r="FG19" s="4" t="n">
-        <v>1.39</v>
+        <v>1.4</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="20">
@@ -8490,7 +8490,7 @@
         <v>8</v>
       </c>
       <c r="FG20" s="4" t="n">
-        <v>1.04</v>
+        <v>1.05</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="21">
@@ -8903,7 +8903,7 @@
         <v>2</v>
       </c>
       <c r="FG21" s="4" t="n">
-        <v>1.07</v>
+        <v>1.08</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="22">
@@ -9334,7 +9334,7 @@
         <v>2</v>
       </c>
       <c r="FG22" s="4" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="23">
@@ -9769,7 +9769,7 @@
         <v>2</v>
       </c>
       <c r="FG23" s="4" t="n">
-        <v>1.41</v>
+        <v>1.42</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="24">
@@ -10427,7 +10427,7 @@
         <v>0</v>
       </c>
       <c r="FG25" s="4" t="n">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="26">
@@ -10760,7 +10760,7 @@
         <v>4</v>
       </c>
       <c r="FG26" s="4" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="27">
@@ -11093,7 +11093,7 @@
         <v>6</v>
       </c>
       <c r="FG27" s="4" t="n">
-        <v>1.04</v>
+        <v>1.06</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="28">
@@ -11514,7 +11514,7 @@
         <v>3</v>
       </c>
       <c r="EW28" s="1" t="n">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="EX28" s="3"/>
       <c r="EY28" s="3" t="n">
@@ -11544,7 +11544,7 @@
         <v>3</v>
       </c>
       <c r="FG28" s="4" t="n">
-        <v>1.15</v>
+        <v>1.16</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="29">
@@ -11764,10 +11764,10 @@
         <v>17</v>
       </c>
       <c r="FF29" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="FG29" s="4" t="n">
-        <v>1.98</v>
+        <v>2.02</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="30">
@@ -12212,7 +12212,7 @@
         <v>181</v>
       </c>
       <c r="EW30" s="1" t="n">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="EX30" s="3"/>
       <c r="EY30" s="3" t="n">
@@ -12239,10 +12239,10 @@
         <v>11</v>
       </c>
       <c r="FF30" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="FG30" s="4" t="n">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="31">
@@ -12459,7 +12459,7 @@
         <v>0</v>
       </c>
       <c r="FG31" s="4" t="n">
-        <v>1.73</v>
+        <v>1.77</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="32">
@@ -12878,7 +12878,7 @@
         <v>2</v>
       </c>
       <c r="FG32" s="4" t="n">
-        <v>1.26</v>
+        <v>1.27</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="33">
@@ -13357,7 +13357,7 @@
         <v>2</v>
       </c>
       <c r="FG33" s="4" t="n">
-        <v>1.52</v>
+        <v>1.53</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="34">
@@ -13806,7 +13806,7 @@
         <v>3</v>
       </c>
       <c r="EW34" s="1" t="n">
-        <v>415</v>
+        <v>384</v>
       </c>
       <c r="EX34" s="3"/>
       <c r="EY34" s="3" t="n">
@@ -13836,7 +13836,7 @@
         <v>2</v>
       </c>
       <c r="FG34" s="4" t="n">
-        <v>1.15</v>
+        <v>1.16</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="35">
@@ -14307,7 +14307,7 @@
         <v>2</v>
       </c>
       <c r="FG35" s="4" t="n">
-        <v>1.53</v>
+        <v>1.54</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="36">
@@ -15253,7 +15253,7 @@
         <v>2</v>
       </c>
       <c r="FG37" s="4" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="38">
@@ -15688,7 +15688,7 @@
         <v>2</v>
       </c>
       <c r="FG38" s="4" t="n">
-        <v>1.53</v>
+        <v>1.54</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="39">
@@ -16159,7 +16159,7 @@
         <v>2</v>
       </c>
       <c r="FG39" s="4" t="n">
-        <v>1.02</v>
+        <v>1.03</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="40">
@@ -16354,7 +16354,7 @@
       <c r="EU40" s="1"/>
       <c r="EV40" s="1"/>
       <c r="EW40" s="1" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="EX40" s="3"/>
       <c r="EY40" s="3" t="n">
@@ -16380,7 +16380,7 @@
         <v>0</v>
       </c>
       <c r="FG40" s="4" t="n">
-        <v>1.08</v>
+        <v>1.09</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="41">
@@ -17149,10 +17149,10 @@
         <v>37</v>
       </c>
       <c r="FF42" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="FG42" s="4" t="n">
-        <v>1.51</v>
+        <v>1.52</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="43">
@@ -17563,7 +17563,7 @@
         <v>2</v>
       </c>
       <c r="FG43" s="4" t="n">
-        <v>1.34</v>
+        <v>1.35</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="44">
@@ -18026,7 +18026,7 @@
         <v>2</v>
       </c>
       <c r="FG44" s="4" t="n">
-        <v>1.25</v>
+        <v>1.26</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="45">
@@ -18494,10 +18494,10 @@
         <v>12</v>
       </c>
       <c r="FF45" s="1" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="FG45" s="4" t="n">
-        <v>1.23</v>
+        <v>1.24</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="46">
@@ -18948,7 +18948,7 @@
         <v>2</v>
       </c>
       <c r="FG46" s="4" t="n">
-        <v>0.6</v>
+        <v>0.61</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="47">
@@ -19427,7 +19427,7 @@
         <v>2</v>
       </c>
       <c r="FG47" s="4" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="48">
@@ -20314,10 +20314,10 @@
         <v>11</v>
       </c>
       <c r="FF49" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="FG49" s="4" t="n">
-        <v>1.09</v>
+        <v>1.1</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="50">
@@ -20581,10 +20581,10 @@
         <v>44</v>
       </c>
       <c r="FF50" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="FG50" s="4" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="51">
@@ -21024,10 +21024,10 @@
         <v>11</v>
       </c>
       <c r="FF51" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="FG51" s="4" t="n">
-        <v>1.07</v>
+        <v>1.08</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="52">
@@ -21380,7 +21380,7 @@
         <v>4</v>
       </c>
       <c r="FG52" s="4" t="n">
-        <v>1.24</v>
+        <v>1.25</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="53">
@@ -21785,7 +21785,7 @@
         <v>35</v>
       </c>
       <c r="EW53" s="1" t="n">
-        <v>647</v>
+        <v>636</v>
       </c>
       <c r="EX53" s="3"/>
       <c r="EY53" s="3" t="n">
@@ -21815,7 +21815,7 @@
         <v>2</v>
       </c>
       <c r="FG53" s="4" t="n">
-        <v>0.8</v>
+        <v>0.81</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="54">
@@ -22250,7 +22250,7 @@
         <v>2</v>
       </c>
       <c r="FG54" s="4" t="n">
-        <v>1.9</v>
+        <v>1.91</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="55">
@@ -22657,7 +22657,7 @@
         <v>2</v>
       </c>
       <c r="FG55" s="4" t="n">
-        <v>1.16</v>
+        <v>1.17</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="56">
@@ -23117,7 +23117,7 @@
         <v>15</v>
       </c>
       <c r="FF56" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="FG56" s="4" t="n">
         <v>0.96</v>
@@ -23583,7 +23583,7 @@
         <v>2</v>
       </c>
       <c r="FG57" s="4" t="n">
-        <v>1.28</v>
+        <v>1.29</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="58">
@@ -23994,7 +23994,7 @@
         <v>4</v>
       </c>
       <c r="EW58" s="1" t="n">
-        <v>598</v>
+        <v>582</v>
       </c>
       <c r="EX58" s="3"/>
       <c r="EY58" s="3" t="n">
@@ -24453,7 +24453,7 @@
         <v>15</v>
       </c>
       <c r="EW59" s="1" t="n">
-        <v>623</v>
+        <v>634</v>
       </c>
       <c r="EX59" s="3"/>
       <c r="EY59" s="3" t="n">
@@ -24483,7 +24483,7 @@
         <v>2</v>
       </c>
       <c r="FG59" s="4" t="n">
-        <v>0.86</v>
+        <v>0.87</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="60">
@@ -24942,7 +24942,7 @@
         <v>2</v>
       </c>
       <c r="FG60" s="4" t="n">
-        <v>1.36</v>
+        <v>1.37</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="61">
@@ -25377,7 +25377,7 @@
         <v>2</v>
       </c>
       <c r="FG61" s="4" t="n">
-        <v>1.06</v>
+        <v>1.07</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="62">
@@ -25808,7 +25808,7 @@
         <v>2</v>
       </c>
       <c r="FG62" s="4" t="n">
-        <v>1.61</v>
+        <v>1.63</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="63">
@@ -26079,7 +26079,7 @@
         <v>13</v>
       </c>
       <c r="FG63" s="4" t="n">
-        <v>0.88</v>
+        <v>0.9</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="64">
@@ -26514,7 +26514,7 @@
         <v>2</v>
       </c>
       <c r="FG64" s="4" t="n">
-        <v>1.08</v>
+        <v>1.09</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="65">
@@ -26967,7 +26967,7 @@
         <v>5</v>
       </c>
       <c r="FG65" s="4" t="n">
-        <v>0.99</v>
+        <v>1</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="66">
@@ -27378,7 +27378,7 @@
         <v>12</v>
       </c>
       <c r="EW66" s="1" t="n">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="EX66" s="3"/>
       <c r="EY66" s="3" t="n">
@@ -27408,7 +27408,7 @@
         <v>3</v>
       </c>
       <c r="FG66" s="4" t="n">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="67">
@@ -27815,7 +27815,7 @@
         <v>2</v>
       </c>
       <c r="FG67" s="4" t="n">
-        <v>1.31</v>
+        <v>1.32</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="68">
@@ -28047,10 +28047,10 @@
         <v>30</v>
       </c>
       <c r="FF68" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="FG68" s="4" t="n">
-        <v>1.84</v>
+        <v>1.87</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="69">
@@ -28487,7 +28487,7 @@
         <v>2</v>
       </c>
       <c r="FG69" s="4" t="n">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="70">
@@ -28950,7 +28950,7 @@
         <v>2</v>
       </c>
       <c r="FG70" s="4" t="n">
-        <v>1.04</v>
+        <v>1.05</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="71">
@@ -29385,7 +29385,7 @@
         <v>3</v>
       </c>
       <c r="FG71" s="4" t="n">
-        <v>1.25</v>
+        <v>1.26</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="72">
@@ -29814,7 +29814,7 @@
         <v>7</v>
       </c>
       <c r="EW72" s="1" t="n">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="EX72" s="3"/>
       <c r="EY72" s="3" t="n">
@@ -30253,7 +30253,7 @@
         <v>7</v>
       </c>
       <c r="EW73" s="1" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="EX73" s="3"/>
       <c r="EY73" s="3" t="n">
@@ -30283,7 +30283,7 @@
         <v>2</v>
       </c>
       <c r="FG73" s="4" t="n">
-        <v>0.49</v>
+        <v>0.5</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="74">
@@ -30756,7 +30756,7 @@
         <v>5</v>
       </c>
       <c r="FG74" s="4" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="75">
@@ -31191,7 +31191,7 @@
         <v>2</v>
       </c>
       <c r="FG75" s="4" t="n">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="76">
@@ -31654,7 +31654,7 @@
         <v>2</v>
       </c>
       <c r="FG76" s="4" t="n">
-        <v>1.13</v>
+        <v>1.14</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="77">
@@ -32089,7 +32089,7 @@
         <v>2</v>
       </c>
       <c r="FG77" s="4" t="n">
-        <v>1.55</v>
+        <v>1.56</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="78">
@@ -32552,7 +32552,7 @@
         <v>3</v>
       </c>
       <c r="FG78" s="4" t="n">
-        <v>1.51</v>
+        <v>1.52</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="79">
@@ -32993,7 +32993,7 @@
         <v>2</v>
       </c>
       <c r="FG79" s="4" t="n">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="80">
@@ -33428,7 +33428,7 @@
         <v>9</v>
       </c>
       <c r="FG80" s="4" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="81">
@@ -33633,7 +33633,7 @@
         <v>100</v>
       </c>
       <c r="FG81" s="4" t="n">
-        <v>1.58</v>
+        <v>1.67</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="82">
@@ -33838,7 +33838,7 @@
         <v>100</v>
       </c>
       <c r="FG82" s="4" t="n">
-        <v>1.97</v>
+        <v>2.13</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="83">
@@ -34277,7 +34277,7 @@
         <v>2</v>
       </c>
       <c r="FG83" s="4" t="n">
-        <v>1.06</v>
+        <v>1.07</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="84">
@@ -34712,7 +34712,7 @@
         <v>2</v>
       </c>
       <c r="FG84" s="4" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="85">
@@ -35586,7 +35586,7 @@
         <v>3</v>
       </c>
       <c r="EW86" s="1" t="n">
-        <v>481</v>
+        <v>474</v>
       </c>
       <c r="EX86" s="3"/>
       <c r="EY86" s="3" t="n">
@@ -35616,7 +35616,7 @@
         <v>3</v>
       </c>
       <c r="FG86" s="4" t="n">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="87">
@@ -36061,7 +36061,7 @@
         <v>4</v>
       </c>
       <c r="EW87" s="1" t="n">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="EX87" s="3"/>
       <c r="EY87" s="3" t="n">
@@ -36091,7 +36091,7 @@
         <v>4</v>
       </c>
       <c r="FG87" s="4" t="n">
-        <v>1.14</v>
+        <v>1.15</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="88">
@@ -36523,7 +36523,7 @@
         <v>16</v>
       </c>
       <c r="FF88" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="FG88" s="4" t="n">
         <v>1.56</v>
@@ -36711,7 +36711,7 @@
       <c r="EU89" s="1"/>
       <c r="EV89" s="1"/>
       <c r="EW89" s="1" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="EX89" s="3"/>
       <c r="EY89" s="3" t="n">
@@ -36737,7 +36737,7 @@
         <v>0</v>
       </c>
       <c r="FG89" s="4" t="n">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="90">
@@ -37585,7 +37585,7 @@
         <v>15</v>
       </c>
       <c r="EW91" s="1" t="n">
-        <v>486</v>
+        <v>497</v>
       </c>
       <c r="EX91" s="3"/>
       <c r="EY91" s="3" t="n">
@@ -38051,7 +38051,7 @@
         <v>16</v>
       </c>
       <c r="FF92" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="FG92" s="4" t="n">
         <v>0.93</v>
@@ -38513,7 +38513,7 @@
         <v>4</v>
       </c>
       <c r="FG93" s="4" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="94">
@@ -38830,7 +38830,7 @@
         <v>13</v>
       </c>
       <c r="FG94" s="4" t="n">
-        <v>1.04</v>
+        <v>1.05</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="95">
@@ -39035,7 +39035,7 @@
         <v>100</v>
       </c>
       <c r="FG95" s="4" t="n">
-        <v>2.08</v>
+        <v>2.17</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="96">
@@ -39440,7 +39440,7 @@
         <v>4</v>
       </c>
       <c r="EW96" s="1" t="n">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="EX96" s="3"/>
       <c r="EY96" s="3" t="n">
@@ -39470,7 +39470,7 @@
         <v>4</v>
       </c>
       <c r="FG96" s="4" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="97">
@@ -40316,7 +40316,7 @@
         <v>4</v>
       </c>
       <c r="FG98" s="4" t="n">
-        <v>1.07</v>
+        <v>1.08</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="99">
@@ -40723,7 +40723,7 @@
         <v>3</v>
       </c>
       <c r="FG99" s="4" t="n">
-        <v>1.42</v>
+        <v>1.43</v>
       </c>
     </row>
     <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="100">
@@ -41040,7 +41040,1318 @@
         <v>21</v>
       </c>
       <c r="FG100" s="4" t="n">
-        <v>0.75</v>
+        <v>0.76</v>
+      </c>
+    </row>
+    <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="101">
+      <c r="A101" s="1" t="n">
+        <v>246</v>
+      </c>
+      <c r="B101" s="2"/>
+      <c r="C101" s="2"/>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>interview</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>fre</t>
+        </is>
+      </c>
+      <c r="G101" s="3" t="n">
+        <v>46224.777511574</v>
+      </c>
+      <c r="H101" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="I101" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="J101" s="2"/>
+      <c r="K101" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="L101" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="M101" s="2"/>
+      <c r="N101" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="O101" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="P101" s="2"/>
+      <c r="Q101" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="R101" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="S101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="T101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="U101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="V101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="W101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="X101" s="1" t="n">
+        <v> -2</v>
+      </c>
+      <c r="Y101" s="2" t="inlineStr">
+        <is>
+          <t>Française</t>
+        </is>
+      </c>
+      <c r="Z101" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="AA101" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="AB101" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="AC101" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="AD101" s="1"/>
+      <c r="AE101" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="AF101" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="AG101" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI101" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT101" s="2"/>
+      <c r="AU101" s="2" t="inlineStr">
+        <is>
+          <t>1967</t>
+        </is>
+      </c>
+      <c r="AV101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX101" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY101" s="2"/>
+      <c r="AZ101" s="2" t="inlineStr">
+        <is>
+          <t>65197</t>
+        </is>
+      </c>
+      <c r="BA101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB101" s="1"/>
+      <c r="BC101" s="1"/>
+      <c r="BD101" s="1"/>
+      <c r="BE101" s="1"/>
+      <c r="BF101" s="1"/>
+      <c r="BG101" s="1"/>
+      <c r="BH101" s="1"/>
+      <c r="BI101" s="1"/>
+      <c r="BJ101" s="1"/>
+      <c r="BK101" s="1"/>
+      <c r="BL101" s="1"/>
+      <c r="BM101" s="1"/>
+      <c r="BN101" s="1"/>
+      <c r="BO101" s="1"/>
+      <c r="BP101" s="1"/>
+      <c r="BQ101" s="1"/>
+      <c r="BR101" s="1"/>
+      <c r="BS101" s="1"/>
+      <c r="BT101" s="1"/>
+      <c r="BU101" s="1"/>
+      <c r="BV101" s="2"/>
+      <c r="BW101" s="1"/>
+      <c r="BX101" s="1"/>
+      <c r="BY101" s="1"/>
+      <c r="BZ101" s="1"/>
+      <c r="CA101" s="1"/>
+      <c r="CB101" s="1"/>
+      <c r="CC101" s="1"/>
+      <c r="CD101" s="1"/>
+      <c r="CE101" s="1"/>
+      <c r="CF101" s="1"/>
+      <c r="CG101" s="1"/>
+      <c r="CH101" s="1"/>
+      <c r="CI101" s="1"/>
+      <c r="CJ101" s="1"/>
+      <c r="CK101" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="CL101" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="CM101" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="CN101" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="CO101" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="CP101" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="CQ101" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="CR101" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="CS101" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="CT101" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="CU101" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="CV101" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="CW101" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="CX101" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="CY101" s="1"/>
+      <c r="CZ101" s="1"/>
+      <c r="DA101" s="1"/>
+      <c r="DB101" s="1"/>
+      <c r="DC101" s="1"/>
+      <c r="DD101" s="1"/>
+      <c r="DE101" s="1"/>
+      <c r="DF101" s="1"/>
+      <c r="DG101" s="1"/>
+      <c r="DH101" s="2"/>
+      <c r="DI101" s="1"/>
+      <c r="DJ101" s="1"/>
+      <c r="DK101" s="1"/>
+      <c r="DL101" s="1"/>
+      <c r="DM101" s="1"/>
+      <c r="DN101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="DO101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="DP101" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="DQ101" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="DR101" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="DS101" s="1"/>
+      <c r="DT101" s="1"/>
+      <c r="DU101" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="DV101" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="DW101" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="DX101" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="DY101" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="DZ101" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="EA101" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="EB101" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="EC101" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="ED101" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="EE101" s="1"/>
+      <c r="EF101" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="EG101" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="EH101" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="EI101" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="EJ101" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="EK101" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="EL101" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="EM101" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="EN101" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="EO101" s="1"/>
+      <c r="EP101" s="1"/>
+      <c r="EQ101" s="1"/>
+      <c r="ER101" s="1"/>
+      <c r="ES101" s="1"/>
+      <c r="ET101" s="1"/>
+      <c r="EU101" s="1"/>
+      <c r="EV101" s="1"/>
+      <c r="EW101" s="1" t="n">
+        <v>227</v>
+      </c>
+      <c r="EX101" s="3"/>
+      <c r="EY101" s="3" t="n">
+        <v>46224.780335648</v>
+      </c>
+      <c r="EZ101" s="2"/>
+      <c r="FA101" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="FB101" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="FC101" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="FD101" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="FE101" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="FF101" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="FG101" s="4" t="n">
+        <v>1.03</v>
+      </c>
+    </row>
+    <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="102">
+      <c r="A102" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="B102" s="2"/>
+      <c r="C102" s="2"/>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>interview</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>ger</t>
+        </is>
+      </c>
+      <c r="G102" s="3" t="n">
+        <v>46240.864953704</v>
+      </c>
+      <c r="H102" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="I102" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="J102" s="2"/>
+      <c r="K102" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="L102" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="M102" s="2"/>
+      <c r="N102" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="O102" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="P102" s="2"/>
+      <c r="Q102" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="R102" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="S102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="T102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="U102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="V102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="W102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="X102" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="Y102" s="2"/>
+      <c r="Z102" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="AA102" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="AB102" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="AC102" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD102" s="1"/>
+      <c r="AE102" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK102" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT102" s="2"/>
+      <c r="AU102" s="2" t="inlineStr">
+        <is>
+          <t>1992</t>
+        </is>
+      </c>
+      <c r="AV102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW102" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="AX102" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY102" s="2"/>
+      <c r="AZ102" s="2" t="inlineStr">
+        <is>
+          <t>55131</t>
+        </is>
+      </c>
+      <c r="BA102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB102" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="BC102" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="BD102" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="BE102" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="BF102" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="BG102" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="BH102" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI102" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="BJ102" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="BK102" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL102" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="BM102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP102" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BS102" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="BT102" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV102" s="2"/>
+      <c r="BW102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BX102" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="BY102" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="BZ102" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="CA102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CB102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CC102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CD102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CE102" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="CF102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CG102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH102" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="CI102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CJ102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CK102" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="CL102" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="CM102" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="CN102" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="CO102" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="CP102" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="CQ102" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="CR102" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="CS102" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="CT102" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="CU102" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="CV102" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="CW102" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="CX102" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="CY102" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="CZ102" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="DA102" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="DB102" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="DC102" s="1"/>
+      <c r="DD102" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="DE102" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="DF102" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="DG102" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="DH102" s="2" t="inlineStr">
+        <is>
+          <t>Man wird nicjt so oft gefragt über die gesamte erlebnis in Deutschland.</t>
+        </is>
+      </c>
+      <c r="DI102" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="DJ102" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="DK102" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="DL102" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="DM102" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="DN102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="DO102" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="DP102" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="DQ102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="DR102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="DS102" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="DT102" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="DU102" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="DV102" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="DW102" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="DX102" s="1" t="n">
+        <v>37</v>
+      </c>
+      <c r="DY102" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="DZ102" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="EA102" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="EB102" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="EC102" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="ED102" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="EE102" s="1"/>
+      <c r="EF102" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="EG102" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="EH102" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="EI102" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="EJ102" s="1" t="n">
+        <v>141</v>
+      </c>
+      <c r="EK102" s="1" t="n">
+        <v>143</v>
+      </c>
+      <c r="EL102" s="1" t="n">
+        <v>101</v>
+      </c>
+      <c r="EM102" s="1" t="n">
+        <v>131</v>
+      </c>
+      <c r="EN102" s="1" t="n">
+        <v>156</v>
+      </c>
+      <c r="EO102" s="1" t="n">
+        <v>89</v>
+      </c>
+      <c r="EP102" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="EQ102" s="1" t="n">
+        <v>328</v>
+      </c>
+      <c r="ER102" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="ES102" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="ET102" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="EU102" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="EV102" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="EW102" s="1" t="n">
+        <v>537</v>
+      </c>
+      <c r="EX102" s="3"/>
+      <c r="EY102" s="3" t="n">
+        <v>46240.884375</v>
+      </c>
+      <c r="EZ102" s="2" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="FA102" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="FB102" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="FC102" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="FD102" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="FE102" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="FF102" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="FG102" s="4" t="n">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row collapsed="false" customFormat="false" customHeight="false" hidden="false" ht="12.1" outlineLevel="0" r="103">
+      <c r="A103" s="1" t="n">
+        <v>251</v>
+      </c>
+      <c r="B103" s="2"/>
+      <c r="C103" s="2"/>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>interview</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>eng</t>
+        </is>
+      </c>
+      <c r="G103" s="3" t="n">
+        <v>46257.214780093</v>
+      </c>
+      <c r="H103" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="I103" s="1" t="n">
+        <v>181</v>
+      </c>
+      <c r="J103" s="2"/>
+      <c r="K103" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="L103" s="1" t="n">
+        <v>181</v>
+      </c>
+      <c r="M103" s="2"/>
+      <c r="N103" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="O103" s="1" t="n">
+        <v>181</v>
+      </c>
+      <c r="P103" s="2"/>
+      <c r="Q103" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="R103" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="S103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="T103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="U103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="V103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="W103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="X103" s="1" t="n">
+        <v> -1</v>
+      </c>
+      <c r="Y103" s="2"/>
+      <c r="Z103" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="AA103" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="AB103" s="1" t="n">
+        <v> -9</v>
+      </c>
+      <c r="AC103" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD103" s="1"/>
+      <c r="AE103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ103" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT103" s="2"/>
+      <c r="AU103" s="2"/>
+      <c r="AV103" s="1" t="n">
+        <v> -1</v>
+      </c>
+      <c r="AW103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX103" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="AY103" s="2"/>
+      <c r="AZ103" s="2"/>
+      <c r="BA103" s="1" t="n">
+        <v> -1</v>
+      </c>
+      <c r="BB103" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="BC103" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="BD103" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="BE103" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="BF103" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="BG103" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="BH103" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI103" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ103" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="BK103" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN103" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="BO103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BS103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BT103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV103" s="2"/>
+      <c r="BW103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="BX103" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="BY103" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="BZ103" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="CA103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CB103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CC103" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="CD103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CE103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CF103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CG103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CJ103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CK103" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="CL103" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="CM103" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="CN103" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="CO103" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="CP103" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="CQ103" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="CR103" s="1" t="n">
+        <v> -1</v>
+      </c>
+      <c r="CS103" s="1" t="n">
+        <v> -1</v>
+      </c>
+      <c r="CT103" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="CU103" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="CV103" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="CW103" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="CX103" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="CY103" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="CZ103" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="DA103" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="DB103" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="DC103" s="1"/>
+      <c r="DD103" s="1" t="n">
+        <v> -1</v>
+      </c>
+      <c r="DE103" s="1" t="n">
+        <v> -1</v>
+      </c>
+      <c r="DF103" s="1" t="n">
+        <v> -1</v>
+      </c>
+      <c r="DG103" s="1" t="n">
+        <v> -1</v>
+      </c>
+      <c r="DH103" s="2" t="inlineStr">
+        <is>
+          <t>There is too much racism especially in my work sector/profession.More rules against descrimination in care work should be implemented.Thank you.</t>
+        </is>
+      </c>
+      <c r="DI103" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="DJ103" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="DK103" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="DL103" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="DM103" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="DN103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="DO103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="DP103" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="DQ103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="DR103" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="DS103" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="DT103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="DU103" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="DV103" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="DW103" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="DX103" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="DY103" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="DZ103" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="EA103" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="EB103" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="EC103" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="ED103" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="EE103" s="1"/>
+      <c r="EF103" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="EG103" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="EH103" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="EI103" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="EJ103" s="1" t="n">
+        <v>58</v>
+      </c>
+      <c r="EK103" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="EL103" s="1" t="n">
+        <v>33</v>
+      </c>
+      <c r="EM103" s="1" t="n">
+        <v>26</v>
+      </c>
+      <c r="EN103" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="EO103" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="EP103" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="EQ103" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="ER103" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="ES103" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="ET103" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="EU103" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="EV103" s="1" t="n">
+        <v>115</v>
+      </c>
+      <c r="EW103" s="1" t="n">
+        <v>529</v>
+      </c>
+      <c r="EX103" s="3"/>
+      <c r="EY103" s="3" t="n">
+        <v>46257.222847222</v>
+      </c>
+      <c r="EZ103" s="2" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="FA103" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="FB103" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="FC103" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="FD103" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="FE103" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="FF103" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="FG103" s="4" t="n">
+        <v>0.72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>